<commit_message>
updated the Test data in csv and excel file
</commit_message>
<xml_diff>
--- a/testData/loginData.xlsx
+++ b/testData/loginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CTV\CTV\CTV\Automation\Selenium\automation-assignment\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DF9C4E-90EA-4ABC-9DC4-9A124B5AA099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD241C0D-28CB-496B-85F5-721D202F964B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
   <si>
     <t>emailAddress</t>
   </si>
@@ -37,9 +37,6 @@
   </si>
   <si>
     <t>Password</t>
-  </si>
-  <si>
-    <t>nimepej425@koboywin.com</t>
   </si>
 </sst>
 </file>
@@ -357,7 +354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -388,18 +385,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{3A734221-6270-4648-A6DC-DF3EEFC0D814}"/>
-    <hyperlink ref="A4" r:id="rId2" xr:uid="{3466F878-B90D-400A-924B-E4DC694063F8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
login data in Excel has been updated.
</commit_message>
<xml_diff>
--- a/testData/loginData.xlsx
+++ b/testData/loginData.xlsx
@@ -3,29 +3,28 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CTV\CTV\CTV\Automation\Selenium\automation-assignment\testData\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD241C0D-28CB-496B-85F5-721D202F964B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{2AF3E03F-DF45-4363-858D-D19042B7C1AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginTestData" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
   <si>
     <t>emailAddress</t>
   </si>
@@ -354,7 +353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -385,9 +384,18 @@
         <v>3</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{3A734221-6270-4648-A6DC-DF3EEFC0D814}"/>
+    <hyperlink ref="A4" r:id="rId2" xr:uid="{50D12F02-302F-478F-8DE7-EBD51439FEC3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>